<commit_message>
Fix Versorgungsausgleich testakte calculations
</commit_message>
<xml_diff>
--- a/testakten/versausgleich-haerte-bgh-schaefer-nuernberg/xlsx/versorgungsausgleich_berechnung_schaefer.xlsx
+++ b/testakten/versausgleich-haerte-bgh-schaefer-nuernberg/xlsx/versorgungsausgleich_berechnung_schaefer.xlsx
@@ -707,15 +707,15 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>12,5000 EP</t>
+          <t>5,2000 EP (ehezeitlich; 12,5000 EP gesamt)</t>
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>96437.5</v>
+        <v>40118</v>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>6,2500 EP</t>
+          <t>2,6000 EP</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -748,7 +748,7 @@
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>140718.75</v>
+        <v>112559</v>
       </c>
     </row>
     <row r="17">
@@ -884,20 +884,20 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>DRV Bund (umgerechnet, ca.)</t>
+          <t>DRV Bund (ehezeitlich, ca.)</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>433.13</v>
+        <v>180.02</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>216.56</v>
+        <v>90.01000000000001</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>216.56</v>
+        <v>90.01000000000001</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>-216.56</v>
+        <v>-90.01000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -907,10 +907,10 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>-959.97</v>
+        <v>-1086.52</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>959.97</v>
+        <v>1086.52</v>
       </c>
     </row>
     <row r="11">

</xml_diff>